<commit_message>
Fix and populate Paket 1 Bahasa Indonesia Quizizz spreadsheet with real questions
</commit_message>
<xml_diff>
--- a/Paket_1_Bahasa_Indonesia_TKA_SD.xlsx
+++ b/Paket_1_Bahasa_Indonesia_TKA_SD.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paket 1 Bahasa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,27 +471,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 1: contoh soal pemahaman teks.</t>
+          <t>Berdasarkan paragraf pertama teks 'Hutan Mangrove: Benteng Alami Pesisir Pantai', fungsi utama akar tunjang pada tanaman mangrove adalah....</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Menghasilkan buah bakau yang dapat dikonsumsi biota laut</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Menahan hantaman ombak, mencegah abrasi, dan merangkap endapan lumpur</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Menyerap cadangan air tawar dari muara sungai secara maksimal</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Mempercepat proses pasang surut air laut di muara pantai</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -502,7 +502,11 @@
       <c r="H2" t="n">
         <v>60</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,27 +516,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 2: contoh soal pemahaman teks.</t>
+          <t>Ide pokok yang terdapat pada paragraf kedua teks informasi di atas adalah....</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Celah akar mangrove tempat berenang ikan ke laut bebas</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Perbandingan luas hutan mangrove dengan hutan hujan tropis</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Manfaat ekologis hutan mangrove bagi biota laut dan penyerapan karbon</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Keanekaragaman jenis udang dan kepiting di pesisir Indonesia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -543,7 +547,11 @@
       <c r="H3" t="n">
         <v>60</v>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,27 +561,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 3: contoh soal pemahaman teks.</t>
+          <t>Makna istilah kata 'abrasi' pada paragraf pertama teks tersebut adalah....</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Penurunan permukaan tanah akibat pemukiman warga pesisir</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Proses pengikisan batuan atau daratan pantai akibat tenaga gelombang laut</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Pencemaran air laut oleh tumpahan limbah industri pabrik</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Penebangan pohon bakau secara liar oleh nelayan lokal</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -584,7 +592,11 @@
       <c r="H4" t="n">
         <v>60</v>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -594,27 +606,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 4: contoh soal pemahaman teks.</t>
+          <t>Berdasarkan bacaan 'Hutan Mangrove: Benteng Alami Pesisir Pantai', manakah pernyataan berikut yang SESUAI dengan isi teks? (Pilihlah lebih dari satu jawaban benar!)  [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Hutan mangrove hanya mampu tumbuh di perairan air tawar yang tenang.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Celah akar mangrove dimanfaatkan hewan laut kecil sebagai tempat berlindung dan berkembang biak.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Kemampuan mangrove menyerap karbon dioksida lebih tinggi dibanding hutan hujan tropis.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Sistem perakaran mangrove berfungsi memperkeruh ekosistem terumbu karang di laut lepas.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -625,7 +637,11 @@
       <c r="H5" t="n">
         <v>60</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -635,27 +651,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 5: contoh soal pemahaman teks.</t>
+          <t>Simpulan yang paling tepat dari keseluruhan isi teks bacaan tersebut adalah....</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Hutan mangrove memiliki peran vital sebagai pelindung fisik pantai, habitat biota laut, dan penyerap karbon bagi bumi.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Biota laut seperti udang dan kepiting tidak dapat hidup apabila tidak ada hutan bakau di muara.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Hutan hujan tropis di daratan sudah tidak mampu menyerap karbon dioksida di atmosfer bumi.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Semua muara sungai di Indonesia harus ditanami pohon mangrove agar air laut tidak pasang.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +682,11 @@
       <c r="H6" t="n">
         <v>60</v>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -676,7 +696,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 6: contoh soal pemahaman teks.</t>
+          <t>Tentukan kebenaran dari setiap pernyataan berikut berdasarkan teks bacaan hutan mangrove!  [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -707,7 +727,11 @@
       <c r="H7" t="n">
         <v>60</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -717,27 +741,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 7: contoh soal pemahaman teks.</t>
+          <t>Apa yang kemungkinan besar akan terjadi pada kawasan pesisir pantai jika seluruh pohon mangrove di tebang habis? Bacalah cerita fiksi berikut dengan cermat untuk menjawab soal nomor 8 sampai 14!
+Kendi Kejujuran Keling
+Di sebuah desa di lereng bukit, hiduplah Keling, seorang anak yatim yang bekerja sebagai pengantar air bersih untuk warga desa. Setiap pagi, Keling memikul dua buah kendi tanah liat yang diikatkan pada sebatang bambu. Salah satu kendi yang dibawanya memiliki sedikit retakan di bagian bawah, sedangkan kendi yang satunya sangat mulus dan utuh.
+Setiap kali tiba di rumah warga, kendi yang retak itu hanya menyisakan setengah air karena airnya merembes di sepanjang jalan setapak. Kendi yang utuh merasa bangga dan sering menyindir kendi retak. Kendi retak pun merasa sangat bersedih karena merasa tidak bisa menjalankan tugasnya dengan sempurna.
+Melihat kesedihan kendinya, Keling tersenyum lembut lalu berkata, "Wahai kendiku, perhatikanlah sisi jalan setapak yang kita lalui setiap pagi. Tanpa kau sadari, air yang menetes dari celah retakanmu telah menyirami benih-benih bunga di sepanjang jalan. Lihatlah sekarang, bunga-bunga liar mekar indah berwarna-warni dan memberi keharuman bagi siapa saja yang lewat. Setiap kekurangan yang kita miliki tetap bisa membawa kebaikan jika disikapi dengan tulus." Mendengar ucapan Keling, kendi retak merasa berlapang dada dan tidak lagi berkecil hati.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Populasi ikan kecil di laut lepas akan bertambah dengan cepat</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Garis pantai akan mengalami erosi dan abrasi parah akibat hantaman ombak</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Terumbu karang di perairan laut akan semakin bersih dan jernih</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Suhu udara di pesisir pantai akan menjadi jauh lebih sejuk</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -748,7 +776,11 @@
       <c r="H8" t="n">
         <v>60</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -758,27 +790,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 8: contoh soal pemahaman teks.</t>
+          <t>Berdasarkan cerita 'Kendi Kejujuran Keling', bagaimana watak tokoh Keling dalam menyikapi kendinya yang retak?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Pemarah dan mudah putus asa</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Bijaksana, sabar, dan penuh rasa syukur</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Sombong dan membanding-bandingkan barang</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Kikir dan tidak peduli terhadap orang lain</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +821,11 @@
       <c r="H9" t="n">
         <v>60</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -799,27 +835,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 9: contoh soal pemahaman teks.</t>
+          <t>Makna ungkapan 'berlapang dada' pada akhir paragraf cerita tersebut adalah....</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Merasa bangga atas kelebihan dirinya</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Ikhlas dan menerima keadaan dengan lapang hati</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Menyerah dan tidak mau lagi bekerja</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Bernapas lega setelah kelelahan memikul kendi</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -830,7 +866,11 @@
       <c r="H10" t="n">
         <v>60</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -840,27 +880,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 10: contoh soal pemahaman teks.</t>
+          <t>Latar tempat dan waktu terjadinya peristiwa dalam cerita fiksi di atas adalah....</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Di tengah hutan belantara pada malam hari</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Di pasar tradisional pada siang hari</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Di jalan setapak desa lereng bukit pada pagi hari</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Di dermaga pelabuhan pada sore hari</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -871,7 +911,11 @@
       <c r="H11" t="n">
         <v>60</v>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -881,27 +925,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 11: contoh soal pemahaman teks.</t>
+          <t>Manakah pernyataan berikut yang menggambarkan situasi konflik dan perasaan tokoh dalam cerita di atas?  [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Kendi yang utuh merasa bangga dan menyindir kekurangan kendi yang retak.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Kendi yang retak merasa sedih dan berkecil hati karena air yang dibawanya berkurang.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Keling membuang kendi retak karena merasa dirugikan saat mengantar air.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Warga desa memarahi Keling karena kendi yang dibawanya meneteskan air.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -912,7 +956,11 @@
       <c r="H12" t="n">
         <v>60</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -922,27 +970,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 12: contoh soal pemahaman teks.</t>
+          <t>Amanat atau pesan moral yang terkandung dalam cerita tersebut adalah....</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Barang yang rusak harus segera dibuang agar tidak menyusahkan orang lain.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Setiap makhluk memiliki kekurangan, namun kekurangan tersebut tetap bisa memberi manfaat jika disikapi dengan tulus.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Kita harus memamerkan kelebihan yang kita miliki agar dihargai oleh sesama.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Jangan pernah bekerja sebagai pengantar air jika hanya memiliki peralatan sederhana.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -953,7 +1001,11 @@
       <c r="H13" t="n">
         <v>60</v>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -963,7 +1015,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 13: contoh soal pemahaman teks.</t>
+          <t>Tentukan kesesuaian dari pernyataan terkait sikap para tokoh dalam cerita 'Kendi Kejujuran Keling'!  [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -994,7 +1046,11 @@
       <c r="H14" t="n">
         <v>60</v>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1004,27 +1060,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 14: contoh soal pemahaman teks.</t>
+          <t>Lawan kata (antonim) dari ungkapan 'berkecil hati' pada cerita di atas adalah....</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Percaya diri</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Rendah diri</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Tinggi hati</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Murah hati</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1035,7 +1091,11 @@
       <c r="H15" t="n">
         <v>60</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1045,27 +1105,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 15: contoh soal pemahaman teks.</t>
+          <t>Penulisan huruf kapital yang tepat sesuai kaidah Ejaan Bahasa Indonesia (EBI) terdapat pada kalimat....</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Pada hari Minggu, paman mengajak kami berlibur ke danau Toba di Sumatera Utara.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Pada hari Minggu, Paman mengajak kami berlibur ke Danau Toba di Sumatera Utara.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Pada hari minggu, paman mengajak kami berlibur ke Danau toba di sumatera utara.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Pada hari Minggu, paman mengajak kami berlibur ke Danau Toba di Sumatera Utara.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1076,7 +1136,11 @@
       <c r="H16" t="n">
         <v>60</v>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1086,27 +1150,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 16: contoh soal pemahaman teks.</t>
+          <t>Perhatikan kalimat percakapan berikut:
+Ibu berkata antarkan kue ini ke rumah Bu Dewi sekarang
+Penggunaan tanda baca yang paling tepat untuk kalimat langsung di atas adalah....</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Ibu berkata; "Antarkan kue ini ke rumah Bu Dewi sekarang?"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Ibu berkata, "Antarkan kue ini ke rumah Bu Dewi sekarang!"</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Ibu berkata: "antarkan kue ini ke rumah bu Dewi sekarang."</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Ibu berkata, "Antarkan kue ini ke rumah Bu Dewi sekarang?"</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1117,7 +1183,11 @@
       <c r="H17" t="n">
         <v>60</v>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1127,27 +1197,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 17: contoh soal pemahaman teks.</t>
+          <t>Kalimat berikut yang seluruh kosakatanya menggunakan kata baku adalah....</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Ayah membeli obat penurun demam di apotek sesuai jadwal dokter.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Ayah membeli obat penurun demam di apotik sesuai jadual dokter.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Ayah membeli obat penurun demam di apotek sesuai jadual dokter.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Ayah membeli obat penurun demam di apotik sesuai jadwal dokter.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1158,7 +1228,11 @@
       <c r="H18" t="n">
         <v>60</v>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1168,27 +1242,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 18: contoh soal pemahaman teks.</t>
+          <t>Perhatikan kalimat-kalimat berikut:
+(1) Semua para siswa-siswa berkumpul di lapangan upacara.
+(2) Siswa kelas enam sedang membersihkan ruang perpustakaan.
+(3) Roni rajin belajar agar supaya mendapat nilai yang memuaskan.
+(4) Ayah membaca surat kabar di teras rumah.
+Manakah kalimat di atas yang termasuk KALIMAT EFEKTIF?  [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  Kalimat (1)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  Kalimat (2)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  Kalimat (3)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  Kalimat (4)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1199,7 +1278,11 @@
       <c r="H19" t="n">
         <v>60</v>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1209,27 +1292,33 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 19: contoh soal pemahaman teks.</t>
+          <t>Perhatikan petunjuk mencuci tangan yang benar berikut:
+(1) Gosok punggung tangan, sela-sela jari, dan bawah kuku secara merata.
+(2) Basahi kedua telapak tangan dengan air bersih yang mengalir.
+(3) Bilas tangan dengan air bersih mengalir hingga tidak ada busa sabun yang tersisa.
+(4) Tuangkan sabun cair secukupnya pada telapak tangan.
+(5) Keringkan tangan menggunakan handuk bersih atau tisu kering.
+Urutan petunjuk mencuci tangan yang benar dan runtut adalah....</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A.  (2) - (4) - (1) - (3) - (5)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B.  (2) - (1) - (4) - (3) - (5)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C.  (4) - (2) - (1) - (3) - (5)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D.  (2) - (4) - (3) - (1) - (5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1240,7 +1329,11 @@
       <c r="H20" t="n">
         <v>60</v>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1250,7 +1343,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[Paket 1] Soal Bahasa 20: contoh soal pemahaman teks.</t>
+          <t>Tentukan kebenaran dari bentukan kata berimbuhan dalam kalimat berikut!  [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1281,7 +1374,11 @@
       <c r="H21" t="n">
         <v>60</v>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pembahasan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>